<commit_message>
call_deepseek.py: remove hardcoded key, use --api-key flag or DEEPSEEK_API_KEY env
</commit_message>
<xml_diff>
--- a/output/原始数据映射表.xlsx
+++ b/output/原始数据映射表.xlsx
@@ -502,7 +502,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>ontology; two-layer ontology model; ontology building method</t>
+          <t>Ontology; Two-layer ontology model; Ontology building method</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>ontology; survey; ontology library</t>
+          <t>Ontology; Survey; Ontology library</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>ontology learning; ontology engineering; ontology learning tools; knowledge discovery</t>
+          <t>Ontology Learning; Ontology Engineering; Ontology Learning Tools; Knowledge Discovery</t>
         </is>
       </c>
     </row>
@@ -654,7 +654,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>ontology engineering; ontology capture; ontology domain</t>
+          <t>Ontology Engineering; Ontology Capture; Ontology Domain</t>
         </is>
       </c>
     </row>
@@ -692,7 +692,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>ontology; ontology mapping; ranking; objective function; ndcg measure</t>
+          <t>ontology; ontology mapping; ranking; objective function; NDCG measure</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>ontology; software engineering; web ontology language (owl)</t>
+          <t>Ontology; Software Engineering; Web Ontology Language (OWL)</t>
         </is>
       </c>
     </row>
@@ -768,7 +768,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>ontology view; ontology inconsistency detection; ontology modularization</t>
+          <t>Ontology View; Ontology Inconsistency Detection; Ontology Modularization</t>
         </is>
       </c>
     </row>
@@ -806,7 +806,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>information system; ontology; web ontology language</t>
+          <t>Information system; ontology; Web Ontology Language</t>
         </is>
       </c>
     </row>
@@ -882,7 +882,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>alignment; chimaera; glue; h-cone; onion; ontology; ontology alignment; ontology mapping; ontology matching; prompt; s-match</t>
+          <t>Alignment; Chimaera; GLUE; H-CONE; ONION; Ontology; Ontology Alignment; Ontology Mapping; Ontology Matching; Prompt; S-Match</t>
         </is>
       </c>
     </row>
@@ -920,7 +920,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>fmea; quality management; model based; ontology-driven; domain ontology; applied ontology; process modelling</t>
+          <t>FMEA; quality management; model based; ontology-driven; domain ontology; applied ontology; process modelling</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>ontology; ontology alignment; ontology matching; ontology mapping; intelligent agent; meaning negotiation</t>
+          <t>Ontology; Ontology Alignment; Ontology Matching; Ontology Mapping; Intelligent Agent; Meaning Negotiation</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>medical ontology; domain ontology; ontology construction; knowledge management</t>
+          <t>Medical ontology; domain ontology; ontology construction; knowledge management</t>
         </is>
       </c>
     </row>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>ontology; ontology construction; patterns; concept extraction</t>
+          <t>Ontology; ontology construction; patterns; concept extraction</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1072,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>ontology; teaching ontology; ontology evaluation; ontology engineering; knowledge engineering</t>
+          <t>Ontology; teaching ontology; ontology evaluation; ontology engineering; knowledge engineering</t>
         </is>
       </c>
     </row>
@@ -1110,7 +1110,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>ontology; web; referent; url; types</t>
+          <t>ontology; Web; referent; URL; types</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1148,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>ontology integration; ontology mapping; interpretation</t>
+          <t>Ontology integration; Ontology mapping; Interpretation</t>
         </is>
       </c>
     </row>
@@ -1186,7 +1186,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>ontology matching; ontology alignment; ontology partition; semantic heterogeneity</t>
+          <t>Ontology matching; Ontology alignment; Ontology partition; Semantic heterogeneity</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>ontology; mapping; survey</t>
+          <t>Ontology; Mapping; Survey</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>ontology transformation; mof-based model transformation</t>
+          <t>Ontology Transformation; MOF-based Model Transformation</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>egovernment domain ontology; ontology reuse; generic top level ontology; ontology selection metrics</t>
+          <t>eGovernment domain ontology; ontology reuse; generic top level ontology; ontology selection metrics</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>biomedical ontologies; semantic web; ontology population; semantic role; knowledge acquisition</t>
+          <t>Biomedical Ontologies; Semantic Web; Ontology population; Semantic role; Knowledge acquisition</t>
         </is>
       </c>
     </row>
@@ -1452,7 +1452,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>semantic web; gene ontology; disease-related information ontology; association rule mining</t>
+          <t>Semantic Web; Gene Ontology; Disease-related information ontology; Association Rule Mining</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1490,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>corpus based ontology evaluation; terminological ontology evaluation; key-concept extraction; ontology building environment</t>
+          <t>Corpus based ontology evaluation; terminological ontology evaluation; key-concept extraction; ontology building environment</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1566,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>ontology; adaptive hypermedia</t>
+          <t>Ontology; Adaptive hypermedia</t>
         </is>
       </c>
     </row>
@@ -1642,7 +1642,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>ontology; semantic web; protege</t>
+          <t>Ontology; Semantic web; Protege</t>
         </is>
       </c>
     </row>
@@ -1718,7 +1718,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>ontology matching; ontology alignment; ontology patterns; naming patterns; ontology refactoring; semantic web</t>
+          <t>Ontology matching; ontology alignment; ontology patterns; naming patterns; ontology refactoring; semantic web</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1794,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>ontology; semantic heterogeneity; semantic similarity; ontology mapping</t>
+          <t>Ontology; Semantic heterogeneity; Semantic similarity; Ontology mapping</t>
         </is>
       </c>
     </row>
@@ -1832,7 +1832,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>human-robot interaction; wikipedia ontology; behavior ontology; ontology alignment</t>
+          <t>Human-Robot Interaction; Wikipedia Ontology; Behavior Ontology; Ontology Alignment</t>
         </is>
       </c>
     </row>
@@ -1870,7 +1870,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>neighbour similarity measure; ontology; semantic web; ontology partitioning; ontology matching</t>
+          <t>Neighbour similarity measure; Ontology; Semantic web; Ontology partitioning; Ontology matching</t>
         </is>
       </c>
     </row>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>semantic web; lbs; domain ontology; ontology constructing; ontology reasoning</t>
+          <t>Semantic Web; LBS; domain ontology; ontology constructing; ontology reasoning</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>ontology; modular; epsilon - connections; ontology construction</t>
+          <t>Ontology; Modular; epsilon - Connections; Ontology construction</t>
         </is>
       </c>
     </row>
@@ -2022,7 +2022,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>ontology change; ontology evolution; ontology mapping; mapping evolution; mapping reconciliation</t>
+          <t>Ontology change; Ontology evolution; Ontology mapping; Mapping evolution; Mapping reconciliation</t>
         </is>
       </c>
     </row>
@@ -2098,7 +2098,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>ontology management system; design principle; functional framework; ontology tool</t>
+          <t>Ontology Management System; Design Principle; Functional Framework; Ontology tool</t>
         </is>
       </c>
     </row>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>ontology learning; learning process improvement; novice modeler</t>
+          <t>Ontology learning; Learning process improvement; Novice modeler</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>ontology knowledge engineering; geo-ontology; hierarchical tree method; ontology building; ontology management</t>
+          <t>Ontology knowledge engineering; geo-ontology; hierarchical tree method; ontology building; ontology management</t>
         </is>
       </c>
     </row>
@@ -2318,7 +2318,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>ontology; probabilistic ontology; video semantic analyses; multi entity bayesian network</t>
+          <t>Ontology; Probabilistic ontology; video semantic analyses; Multi Entity Bayesian Network</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>ontology; software engineering; sufism</t>
+          <t>Ontology; Software engineering; Sufism</t>
         </is>
       </c>
     </row>
@@ -2394,7 +2394,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>discrete particle swarm optimisation; ontology alignment; ontology mapping; ontology matching; semantic integration; semantic web</t>
+          <t>Discrete particle swarm optimisation; Ontology alignment; Ontology mapping; Ontology matching; Semantic integration; Semantic Web</t>
         </is>
       </c>
     </row>
@@ -2470,7 +2470,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>ontology; meta-ontology; knowledge repositories; knowledge objects; architectural ontologies</t>
+          <t>Ontology; meta-ontology; knowledge repositories; knowledge objects; Architectural Ontologies</t>
         </is>
       </c>
     </row>
@@ -2546,7 +2546,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>ontology; metrics; swoogle; ontorank</t>
+          <t>Ontology; Metrics; Swoogle; OntoRank</t>
         </is>
       </c>
     </row>
@@ -2584,7 +2584,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>geospatial information integration; ontology; ontology matching; information theory</t>
+          <t>Geospatial Information integration; Ontology; Ontology Matching; Information theory</t>
         </is>
       </c>
     </row>
@@ -2622,7 +2622,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>visualization; ontology engineering; flexactionscript</t>
+          <t>Visualization; Ontology Engineering; FlexActionScript</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>data quality; financial decision-making; ontology; ontology mapping; portfolio management</t>
+          <t>Data quality; Financial decision-making; Ontology; Ontology mapping; Portfolio management</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2698,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>interoperability; knowledge verification; foundation ontologies; domain ontologies; common logic</t>
+          <t>Interoperability; Knowledge verification; Foundation ontologies; Domain ontologies; Common Logic</t>
         </is>
       </c>
     </row>
@@ -2736,7 +2736,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>ontology; ontology learning; semantic web; concept extraction; relation extraction</t>
+          <t>ontology; ontology learning; semantic Web; concept extraction; relation extraction</t>
         </is>
       </c>
     </row>
@@ -2812,7 +2812,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>distributed ontology; ontology inconsistency; semantic wiki</t>
+          <t>Distributed Ontology; Ontology Inconsistency; Semantic Wiki</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>substation; ontology; owl</t>
+          <t>Substation; Ontology; OWL</t>
         </is>
       </c>
     </row>
@@ -2888,7 +2888,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>relational databases; ontologies; ontology-based databases</t>
+          <t>Relational databases; Ontologies; Ontology-based databases</t>
         </is>
       </c>
     </row>
@@ -2926,7 +2926,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>ontology engineering; ontology enrichment; owl</t>
+          <t>Ontology Engineering; Ontology Enrichment; OWL</t>
         </is>
       </c>
     </row>
@@ -2964,7 +2964,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>diseases; ontology; swrl; information systems</t>
+          <t>Diseases; Ontology; SWRL; Information systems</t>
         </is>
       </c>
     </row>
@@ -3002,7 +3002,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>sensor ontology; sensor core ontology building; sensor ontology update and extension; semantic sensor web; sensor discovery</t>
+          <t>Sensor Ontology; Sensor Core Ontology Building; Sensor Ontology Update and Extension; Semantic Sensor Web; Sensor Discovery</t>
         </is>
       </c>
     </row>
@@ -3040,7 +3040,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>semantic social networks; ontology distance; ontology similarity; personal ontologies; experimental methodology</t>
+          <t>Semantic social networks; ontology distance; ontology similarity; personal ontologies; experimental methodology</t>
         </is>
       </c>
     </row>
@@ -3078,7 +3078,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>classification; informatics; ontology</t>
+          <t>Classification; Informatics; Ontology</t>
         </is>
       </c>
     </row>
@@ -3116,7 +3116,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>ontology; protege 2000; risk identification</t>
+          <t>ontology; Protege 2000; risk identification</t>
         </is>
       </c>
     </row>
@@ -3154,7 +3154,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>ontology; intellectual property rights (ipr); copyright protection; ontology web language (owl)</t>
+          <t>Ontology; Intellectual property rights (IPR); Copyright protection; Ontology Web Language (OWL)</t>
         </is>
       </c>
     </row>
@@ -3192,7 +3192,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>ontology; ontology meta-data model; knowledge ontology; structural knowledge; extended entity relationship model</t>
+          <t>Ontology; Ontology meta-data model; Knowledge ontology; Structural knowledge; Extended entity relationship model</t>
         </is>
       </c>
     </row>
@@ -3230,7 +3230,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>ontology; semantic search; neuroscience ontologies</t>
+          <t>Ontology; semantic search; neuroscience ontologies</t>
         </is>
       </c>
     </row>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>probabilistic reasoning; ontology queries</t>
+          <t>Probabilistic reasoning; Ontology queries</t>
         </is>
       </c>
     </row>
@@ -3306,7 +3306,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>concept lattice; granular computing; ontology building; ontology merging; ontology connection</t>
+          <t>Concept lattice; Granular computing; Ontology building; Ontology merging; Ontology connection</t>
         </is>
       </c>
     </row>
@@ -3344,7 +3344,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>retrieval; ontology; domain; management</t>
+          <t>Retrieval; Ontology; Domain; Management</t>
         </is>
       </c>
     </row>
@@ -3382,7 +3382,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>ontology matching; integration; context reasoning; knowledge and information integration</t>
+          <t>ontology matching; Integration; context reasoning; knowledge and information integration</t>
         </is>
       </c>
     </row>
@@ -3420,7 +3420,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>ontology; interoperability; data sharing; terms representation; diagnostic systems</t>
+          <t>Ontology; Interoperability; Data sharing; Terms representation; Diagnostic systems</t>
         </is>
       </c>
     </row>
@@ -3458,7 +3458,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>ontologies; knowledge representation; automated reasoning; quality assurance; owl</t>
+          <t>Ontologies; Knowledge representation; Automated reasoning; Quality assurance; OWL</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>herbal medicine; semantic technology; knowledge representation; ontology modeling; ontology engineering</t>
+          <t>Herbal Medicine; Semantic Technology; Knowledge Representation; Ontology Modeling; Ontology Engineering</t>
         </is>
       </c>
     </row>
@@ -3534,7 +3534,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>domain ontology; knowledge engineering; natural language processing; ontology construction; medical ontology</t>
+          <t>Domain ontology; Knowledge engineering; Natural language processing; Ontology construction; Medical ontology</t>
         </is>
       </c>
     </row>
@@ -3572,7 +3572,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>ubiquitous computing; service ontology; ontology structure; evaluation metric; soa</t>
+          <t>Ubiquitous computing; Service ontology; Ontology structure; Evaluation metric; SOA</t>
         </is>
       </c>
     </row>
@@ -3610,7 +3610,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>user profiles; ontology; ole; personalised ontology</t>
+          <t>User profiles; Ontology; OLE; Personalised ontology</t>
         </is>
       </c>
     </row>
@@ -3648,7 +3648,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>relational database; owl; semantic web; ontology; owl view; reverse engineering; ontology learning</t>
+          <t>Relational Database; OWL; Semantic Web; Ontology; OWL View; Reverse Engineering; Ontology Learning</t>
         </is>
       </c>
     </row>
@@ -3724,7 +3724,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>relational database (rdb); schema; ontology; automated ontology construction</t>
+          <t>Relational database (RDB); Schema; Ontology; Automated ontology construction</t>
         </is>
       </c>
     </row>
@@ -3754,7 +3754,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>ontology; systems; big data; engineering; ontological analysis; model; quality</t>
+          <t>Ontology; systems; big data; engineering; ontological analysis; model; quality</t>
         </is>
       </c>
     </row>
@@ -3792,7 +3792,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>domain-driven data mining; ontology; tddmf; data ontology</t>
+          <t>Domain-driven data mining; Ontology; TDDMF; Data ontology</t>
         </is>
       </c>
     </row>
@@ -3830,7 +3830,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>ontology; 5w1h; event model; ontology population</t>
+          <t>Ontology; 5W1H; Event Model; Ontology Population</t>
         </is>
       </c>
     </row>
@@ -3868,7 +3868,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>ontology usage; web of data; ontology usage network</t>
+          <t>Ontology Usage; Web of Data; Ontology Usage Network</t>
         </is>
       </c>
     </row>
@@ -3936,7 +3936,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>ontology building; ontology maintenance; ontology integration; semantic modeling; ontology-based systems</t>
+          <t>Ontology building; ontology maintenance; ontology integration; semantic modeling; ontology-based systems</t>
         </is>
       </c>
     </row>
@@ -4012,7 +4012,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>ontologies; business decision support; semantic web services; ontology similarity assessment; ontology matching</t>
+          <t>Ontologies; Business decision support; Semantic web services; Ontology similarity assessment; Ontology matching</t>
         </is>
       </c>
     </row>
@@ -4050,7 +4050,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>ontology; semantics-based recommendation; heuristics</t>
+          <t>Ontology; Semantics-Based Recommendation; Heuristics</t>
         </is>
       </c>
     </row>
@@ -4088,7 +4088,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>event; event class; event ontology model; event ontology reasoning</t>
+          <t>Event; Event class; Event ontology model; Event ontology reasoning</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>semantic model; ontology web language; spatial temporal; geographical ontology</t>
+          <t>Semantic Model; Ontology Web Language; Spatial Temporal; Geographical Ontology</t>
         </is>
       </c>
     </row>
@@ -4164,7 +4164,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>identifiers; compound keys; reengineering; ontologies</t>
+          <t>Identifiers; Compound keys; Reengineering; Ontologies</t>
         </is>
       </c>
     </row>
@@ -4202,7 +4202,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>ontology matching; probabilistic reasoning; markov networks</t>
+          <t>Ontology matching; Probabilistic reasoning; Markov networks</t>
         </is>
       </c>
     </row>
@@ -4240,7 +4240,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>ontology matching; knowledge integration; software tools</t>
+          <t>Ontology Matching; Knowledge Integration; Software Tools</t>
         </is>
       </c>
     </row>
@@ -4278,7 +4278,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>context-aware; owl; ontology model</t>
+          <t>Context-aware; OWL; ontology model</t>
         </is>
       </c>
     </row>
@@ -4316,7 +4316,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>ontology sharing; web services; biomedical ontology; viral hepatitis ontology; viral hepatitis diagnosis</t>
+          <t>Ontology sharing; Web Services; Biomedical Ontology; Viral Hepatitis Ontology; Viral Hepatitis Diagnosis</t>
         </is>
       </c>
     </row>
@@ -4392,7 +4392,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>ontology; e-learning; reusable; framework</t>
+          <t>ontology; e-Learning; reusable; framework</t>
         </is>
       </c>
     </row>
@@ -4430,7 +4430,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>ontology; ontology integration; ontology matching; ontology alignment; concept importance; concept type and priorly matchable concept</t>
+          <t>Ontology; Ontology integration; Ontology matching; Ontology alignment; Concept importance; Concept type and priorly matchable concept</t>
         </is>
       </c>
     </row>
@@ -4460,7 +4460,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>evaluation; qfd; service-oriented ontology; hoq frame of ontology</t>
+          <t>evaluation; QFD; Service-oriented ontology; HoQ Frame of Ontology</t>
         </is>
       </c>
     </row>
@@ -4498,7 +4498,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>collaborative ontology editing; agricultural ontology; acsw; collaborative protege; webprotege</t>
+          <t>collaborative ontology editing; agricultural ontology; ACSW; Collaborative Protege; WebProtege</t>
         </is>
       </c>
     </row>
@@ -4574,7 +4574,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>enterprise modelling; contracts; ontology; perdurantism</t>
+          <t>Enterprise Modelling; Contracts; Ontology; Perdurantism</t>
         </is>
       </c>
     </row>
@@ -4612,7 +4612,7 @@
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>machine learning; ontology; umls</t>
+          <t>Machine Learning; Ontology; UMLS</t>
         </is>
       </c>
     </row>
@@ -4650,7 +4650,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>activity recognition; context-aware infrastructure ontology; ontology based activity recognition; semantic ontology search</t>
+          <t>Activity recognition; Context-aware infrastructure ontology; Ontology based activity recognition; Semantic ontology search</t>
         </is>
       </c>
     </row>
@@ -4726,7 +4726,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>gesture; speech; reference; ontology</t>
+          <t>Gesture; Speech; Reference; Ontology</t>
         </is>
       </c>
     </row>
@@ -4916,7 +4916,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>ontology; embedded system; epd</t>
+          <t>Ontology; embedded system; EPD</t>
         </is>
       </c>
     </row>
@@ -4954,7 +4954,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>educational information system; erp; semantic web; ontology</t>
+          <t>Educational Information System; ERP; semantic web; ontology</t>
         </is>
       </c>
     </row>
@@ -4992,7 +4992,7 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>fuzzy ontology; fuzzy reasoning; knowledge mobilisation</t>
+          <t>Fuzzy ontology; Fuzzy reasoning; Knowledge mobilisation</t>
         </is>
       </c>
     </row>
@@ -5030,7 +5030,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>ontology; maintenance systems integration; semantic interoperability</t>
+          <t>Ontology; maintenance systems integration; semantic interoperability</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>ontology engineering; ontology economics; cost estimation; planning and controlling</t>
+          <t>Ontology engineering; Ontology economics; Cost estimation; Planning and controlling</t>
         </is>
       </c>
     </row>
@@ -5106,7 +5106,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>ontology annotation; question generation; ontology evolution; egovernment dataset</t>
+          <t>ontology annotation; question generation; ontology evolution; eGovernment dataset</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>ontologies; terminologies; thesauri</t>
+          <t>Ontologies; terminologies; thesauri</t>
         </is>
       </c>
     </row>
@@ -5258,7 +5258,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>semantic web; foaf; persona; vocabulary; ontology</t>
+          <t>Semantic Web; FOAF; Persona; Vocabulary; Ontology</t>
         </is>
       </c>
     </row>
@@ -5296,7 +5296,7 @@
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>multi-perspective; ontology; requirements elicitation</t>
+          <t>Multi-Perspective; Ontology; Requirements Elicitation</t>
         </is>
       </c>
     </row>
@@ -5334,7 +5334,7 @@
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>mass customization; scenario; ontology; requirements</t>
+          <t>Mass Customization; Scenario; Ontology; Requirements</t>
         </is>
       </c>
     </row>
@@ -5372,7 +5372,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>ontology; steel house; 3d; pattern; component</t>
+          <t>ontology; Steel House; 3D; Pattern; Component</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>ontology learning; encyclopedia; concept; taxonomy; instance</t>
+          <t>ontology learning; encyclopedia; concept; taxonomy; Instance</t>
         </is>
       </c>
     </row>
@@ -5486,7 +5486,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>web service clustering; ontology learning</t>
+          <t>Web service clustering; Ontology Learning</t>
         </is>
       </c>
     </row>
@@ -5524,7 +5524,7 @@
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>semantic annotation; ontology mapping; ontology reasoning; swrl</t>
+          <t>Semantic annotation; ontology mapping; ontology reasoning; SWRL</t>
         </is>
       </c>
     </row>
@@ -5554,7 +5554,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>software engineering; it competence; ontology; competency ontology; competency register</t>
+          <t>software engineering; IT competence; ontology; competency ontology; competency register</t>
         </is>
       </c>
     </row>
@@ -5584,7 +5584,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>ontology; thesaurus; semantic web; information retrieval</t>
+          <t>Ontology; thesaurus; semantic web; information retrieval</t>
         </is>
       </c>
     </row>
@@ -5622,7 +5622,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>process supervision; expert systems; ontology</t>
+          <t>Process Supervision; Expert Systems; Ontology</t>
         </is>
       </c>
     </row>
@@ -5660,7 +5660,7 @@
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>knowlegde management systems; ontology; visual representation; semantic; memoria-mea</t>
+          <t>Knowlegde management systems; Ontology; Visual representation; Semantic; Memoria-Mea</t>
         </is>
       </c>
     </row>
@@ -5736,7 +5736,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>city logistics; ontology; agent-based modeling</t>
+          <t>City logistics; Ontology; Agent-based modeling</t>
         </is>
       </c>
     </row>
@@ -5774,7 +5774,7 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>semantic web; ontology; protege 4.0</t>
+          <t>Semantic Web; Ontology; Protege 4.0</t>
         </is>
       </c>
     </row>
@@ -5850,7 +5850,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>controlled natural languages; ontology verbalisation; multilingualism; ontology lexicalisation; natural language generation</t>
+          <t>Controlled Natural Languages; Ontology Verbalisation; Multilingualism; Ontology Lexicalisation; Natural Language Generation</t>
         </is>
       </c>
     </row>
@@ -5926,7 +5926,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>process ontology; emergence; representation; self; values; social ontology; persons; personality; self directedness</t>
+          <t>Process ontology; Emergence; Representation; Self; Values; Social ontology; Persons; Personality; Self directedness</t>
         </is>
       </c>
     </row>
@@ -5964,7 +5964,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>ontology alignment; semantic similarity; fuzzy set similarity; ontology alignment evaluation initiative (oaei)</t>
+          <t>ontology alignment; semantic similarity; fuzzy set similarity; ontology alignment evaluation initiative (OAEI)</t>
         </is>
       </c>
     </row>
@@ -6002,7 +6002,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>folksonomies; ontologies; evaluation; hierarchy quality</t>
+          <t>Folksonomies; Ontologies; Evaluation; Hierarchy quality</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>ontology; knowledge extraction; data mining; influence rules; frequent items</t>
+          <t>Ontology; knowledge extraction; data mining; influence rules; frequent items</t>
         </is>
       </c>
     </row>
@@ -6108,7 +6108,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>robotics; ontologies; methodologies</t>
+          <t>Robotics; ontologies; methodologies</t>
         </is>
       </c>
     </row>
@@ -6146,7 +6146,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>network course; ontology; knowledge point</t>
+          <t>Network Course; Ontology; Knowledge Point</t>
         </is>
       </c>
     </row>
@@ -6184,7 +6184,7 @@
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>lexicon; lexical database; ontologies; semantics; wordnet</t>
+          <t>Lexicon; Lexical Database; Ontologies; Semantics; WordNet</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>ontology; ontology-based retrieval system; intelligent spider program; image retrieval engine</t>
+          <t>Ontology; Ontology-based Retrieval System; Intelligent spider program; Image Retrieval engine</t>
         </is>
       </c>
     </row>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>mammography ontology; case-based retrieval; ontology; sqwrl; breast cancer</t>
+          <t>Mammography ontology; Case-based Retrieval; Ontology; SQWRL; Breast cancer</t>
         </is>
       </c>
     </row>
@@ -6404,7 +6404,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>authority data; relationship ontology; cultural heritage; digital libraries</t>
+          <t>Authority Data; Relationship Ontology; Cultural Heritage; Digital Libraries</t>
         </is>
       </c>
     </row>
@@ -6442,7 +6442,7 @@
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>ontology development; owl; bio-ontology; diagram; pathway; bfo</t>
+          <t>Ontology development; OWL; Bio-ontology; Diagram; Pathway; BFO</t>
         </is>
       </c>
     </row>
@@ -6480,7 +6480,7 @@
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>smart home; home service; domain ontology; need; function</t>
+          <t>Smart Home; Home Service; Domain Ontology; Need; Function</t>
         </is>
       </c>
     </row>
@@ -6556,7 +6556,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>web information extraction; ontology; dom (document object model)</t>
+          <t>Web information extraction; Ontology; DOM (Document Object Model)</t>
         </is>
       </c>
     </row>
@@ -6594,7 +6594,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>ontology; semantic; imagery; video; intelligence; fusion; uav</t>
+          <t>Ontology; semantic; imagery; video; intelligence; fusion; UAV</t>
         </is>
       </c>
     </row>
@@ -6632,7 +6632,7 @@
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>image retrieval; ontology; semantic image; image understanding; semantic retrieval</t>
+          <t>Image Retrieval; Ontology; Semantic Image; Image Understanding; Semantic Retrieval</t>
         </is>
       </c>
     </row>
@@ -6670,7 +6670,7 @@
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>ontology; ontology learning; non-taxonomic relationships; natural language processing</t>
+          <t>Ontology; Ontology learning; Non-taxonomic relationships; Natural Language Processing</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>semantic web; ontology; search; semantic similarity</t>
+          <t>Semantic Web; Ontology; Search; Semantic similarity</t>
         </is>
       </c>
     </row>
@@ -6746,7 +6746,7 @@
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>semantic web; intelligent web; ontology design; swoop; semantic search patterns; kim</t>
+          <t>Semantic Web; Intelligent Web; Ontology Design; Swoop; Semantic Search patterns; KIM</t>
         </is>
       </c>
     </row>
@@ -6784,7 +6784,7 @@
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>ontology; structuring; chaos; fibrils; microvolumes; microvacuoles; matter; neodarwinism</t>
+          <t>Ontology; Structuring; Chaos; Fibrils; Microvolumes; Microvacuoles; Matter; NeoDarwinism</t>
         </is>
       </c>
     </row>
@@ -6852,7 +6852,7 @@
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>precision agriculture; ontology; knowledge presentation</t>
+          <t>Precision Agriculture; Ontology; knowledge presentation</t>
         </is>
       </c>
     </row>
@@ -6890,7 +6890,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>tag clouds; ontologies; semantic networks; wordnet</t>
+          <t>Tag clouds; ontologies; semantic networks; WordNet</t>
         </is>
       </c>
     </row>
@@ -6928,7 +6928,7 @@
       </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>ontology matching; benchmarking; multilingualism; data integration</t>
+          <t>Ontology matching; Benchmarking; Multilingualism; Data integration</t>
         </is>
       </c>
     </row>
@@ -6966,7 +6966,7 @@
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>arabic expansion; wordnet ontology; ontology expansion; information retrieval</t>
+          <t>Arabic expansion; WordNet Ontology; Ontology Expansion; Information Retrieval</t>
         </is>
       </c>
     </row>
@@ -7072,7 +7072,7 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>pattern; knowledge fusion; ontology alignment</t>
+          <t>Pattern; knowledge fusion; ontology alignment</t>
         </is>
       </c>
     </row>
@@ -7110,7 +7110,7 @@
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>ontology mapping; entropy; decision-making</t>
+          <t>ontology mapping; Entropy; decision-making</t>
         </is>
       </c>
     </row>
@@ -7148,7 +7148,7 @@
       </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>ontology; organizational learning; learning organization</t>
+          <t>Ontology; Organizational learning; Learning organization</t>
         </is>
       </c>
     </row>
@@ -7224,7 +7224,7 @@
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>decision-making; knowledge modeling; ontology</t>
+          <t>Decision-Making; Knowledge Modeling; Ontology</t>
         </is>
       </c>
     </row>
@@ -7262,7 +7262,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>domain ontology; methodology; software engineering</t>
+          <t>Domain Ontology; Methodology; Software Engineering</t>
         </is>
       </c>
     </row>
@@ -7338,7 +7338,7 @@
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>ontology; diagnostics system; self-diagnostic device; maintenance</t>
+          <t>Ontology; diagnostics system; self-diagnostic device; maintenance</t>
         </is>
       </c>
     </row>
@@ -7376,7 +7376,7 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>ontologies; owl; class classification; property classification; optimisations</t>
+          <t>Ontologies; OWL; Class classification; Property classification; Optimisations</t>
         </is>
       </c>
     </row>
@@ -7414,7 +7414,7 @@
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>terminology; ontology; distinction; entities; relations; knowledge; continuum</t>
+          <t>Terminology; ontology; distinction; entities; relations; knowledge; continuum</t>
         </is>
       </c>
     </row>
@@ -7452,7 +7452,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>production performance indicators; ontology; classification</t>
+          <t>Production Performance Indicators; Ontology; Classification</t>
         </is>
       </c>
     </row>
@@ -7490,7 +7490,7 @@
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>clinical pathways; ontology; semantic rules; emr</t>
+          <t>Clinical pathways; Ontology; Semantic rules; EMR</t>
         </is>
       </c>
     </row>
@@ -7566,7 +7566,7 @@
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>ontologies; neuroimaging; cognitive experiments; brain mapping</t>
+          <t>Ontologies; Neuroimaging; Cognitive experiments; Brain mapping</t>
         </is>
       </c>
     </row>
@@ -7642,7 +7642,7 @@
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>mri; artifact; ontology; image</t>
+          <t>MRI; Artifact; Ontology; Image</t>
         </is>
       </c>
     </row>
@@ -7680,7 +7680,7 @@
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>events; models; principles; pattern-oriented ontology design; core ontologies</t>
+          <t>Events; Models; Principles; Pattern-oriented ontology design; Core ontologies</t>
         </is>
       </c>
     </row>
@@ -7718,7 +7718,7 @@
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>ontology instance matching; record linkage; semantic knowledge base; ontology alignment; ontology population; identity recognition; linked data; anchor-flood algorithm</t>
+          <t>Ontology Instance Matching; Record Linkage; Semantic Knowledge base; Ontology alignment; Ontology Population; Identity Recognition; Linked Data; Anchor-flood Algorithm</t>
         </is>
       </c>
     </row>
@@ -7756,7 +7756,7 @@
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>ontology; agricultural ontology service (aos); agricultural pest; metadata collection</t>
+          <t>ontology; agricultural ontology service (AOS); agricultural pest; metadata collection</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>role; ontology; owl; disjoint set; social network</t>
+          <t>Role; Ontology; OWL; Disjoint set; Social Network</t>
         </is>
       </c>
     </row>
@@ -7832,7 +7832,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>bfo; ontoclean; ontology</t>
+          <t>BFO; OntoClean; ontology</t>
         </is>
       </c>
     </row>
@@ -7870,7 +7870,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>brief ontology; knowledge representation; knowledge mobilization; environmental impact assessment</t>
+          <t>Brief ontology; Knowledge representation; Knowledge mobilization; Environmental impact assessment</t>
         </is>
       </c>
     </row>
@@ -7908,7 +7908,7 @@
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>ontology of time; time point; time interval; coincidence; brentano</t>
+          <t>Ontology of Time; Time Point; Time Interval; Coincidence; Brentano</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7946,7 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>security; ontologies; requirements; analysis; classification</t>
+          <t>Security; Ontologies; Requirements; Analysis; Classification</t>
         </is>
       </c>
     </row>
@@ -7984,7 +7984,7 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>ontology; adaptive learning; user model; user context; learning activity</t>
+          <t>ontology; Adaptive learning; user model; user context; learning activity</t>
         </is>
       </c>
     </row>

</xml_diff>